<commit_message>
[v6.4.2]DL PEDCA and light load scenario added
</commit_message>
<xml_diff>
--- a/delay_pdf/11be/fix_nsta30_CwdsxQSRCxPSRC_sweep/param_p99_heatmap_1Mbps.xlsx
+++ b/delay_pdf/11be/fix_nsta30_CwdsxQSRCxPSRC_sweep/param_p99_heatmap_1Mbps.xlsx
@@ -560,29 +560,17 @@
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n">
-        <v>9102</v>
-      </c>
-      <c r="C5" s="6" t="n">
-        <v>11502</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>9652</v>
-      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
-        <v>9102</v>
-      </c>
-      <c r="H5" s="6" t="n">
-        <v>11232</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>10808</v>
-      </c>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -590,29 +578,17 @@
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n">
-        <v>9498</v>
-      </c>
-      <c r="C6" s="6" t="n">
-        <v>11538</v>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>9952</v>
-      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
       <c r="F6" s="5" t="inlineStr">
         <is>
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="G6" s="6" t="n">
-        <v>10172</v>
-      </c>
-      <c r="H6" s="6" t="n">
-        <v>8272</v>
-      </c>
-      <c r="I6" s="6" t="n">
-        <v>10068</v>
-      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
@@ -620,29 +596,17 @@
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="B7" s="6" t="n">
-        <v>10982</v>
-      </c>
-      <c r="C7" s="6" t="n">
-        <v>10892</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>10172</v>
-      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
-        <v>8258</v>
-      </c>
-      <c r="H7" s="6" t="n">
-        <v>11488</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>10542</v>
-      </c>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -650,29 +614,17 @@
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="B8" s="6" t="n">
-        <v>10788</v>
-      </c>
-      <c r="C8" s="6" t="n">
-        <v>8492</v>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>9142</v>
-      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
       <c r="F8" s="5" t="inlineStr">
         <is>
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="G8" s="6" t="n">
-        <v>10798</v>
-      </c>
-      <c r="H8" s="6" t="n">
-        <v>10222</v>
-      </c>
-      <c r="I8" s="6" t="n">
-        <v>9888</v>
-      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -680,29 +632,17 @@
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="B9" s="6" t="n">
-        <v>8812</v>
-      </c>
-      <c r="C9" s="6" t="n">
-        <v>8388</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>9798</v>
-      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
       <c r="F9" s="5" t="inlineStr">
         <is>
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
-        <v>9842</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>9232</v>
-      </c>
-      <c r="I9" s="6" t="n">
-        <v>10318</v>
-      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -710,29 +650,17 @@
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n">
-        <v>10092</v>
-      </c>
-      <c r="C10" s="6" t="n">
-        <v>10872</v>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>10472</v>
-      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
       <c r="F10" s="5" t="inlineStr">
         <is>
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="G10" s="6" t="n">
-        <v>9702</v>
-      </c>
-      <c r="H10" s="6" t="n">
-        <v>9792</v>
-      </c>
-      <c r="I10" s="6" t="n">
-        <v>10568</v>
-      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -789,29 +717,17 @@
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n">
-        <v>10408</v>
-      </c>
-      <c r="C14" s="6" t="n">
-        <v>10232</v>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>8178</v>
-      </c>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
       <c r="F14" s="5" t="inlineStr">
         <is>
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="G14" s="6" t="n">
-        <v>10408</v>
-      </c>
-      <c r="H14" s="6" t="n">
-        <v>9152</v>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>8292</v>
-      </c>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -819,29 +735,17 @@
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="B15" s="6" t="n">
-        <v>9578</v>
-      </c>
-      <c r="C15" s="6" t="n">
-        <v>8752</v>
-      </c>
-      <c r="D15" s="6" t="n">
-        <v>9048</v>
-      </c>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="G15" s="6" t="n">
-        <v>10048</v>
-      </c>
-      <c r="H15" s="6" t="n">
-        <v>9918</v>
-      </c>
-      <c r="I15" s="6" t="n">
-        <v>9698</v>
-      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -849,29 +753,17 @@
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="B16" s="6" t="n">
-        <v>9048</v>
-      </c>
-      <c r="C16" s="6" t="n">
-        <v>8712</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>8622</v>
-      </c>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
       <c r="F16" s="5" t="inlineStr">
         <is>
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="G16" s="6" t="n">
-        <v>11012</v>
-      </c>
-      <c r="H16" s="6" t="n">
-        <v>8392</v>
-      </c>
-      <c r="I16" s="6" t="n">
-        <v>9358</v>
-      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -879,29 +771,17 @@
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n">
-        <v>9408</v>
-      </c>
-      <c r="C17" s="6" t="n">
-        <v>11408</v>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>10382</v>
-      </c>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
       <c r="F17" s="5" t="inlineStr">
         <is>
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="G17" s="6" t="n">
-        <v>9732</v>
-      </c>
-      <c r="H17" s="6" t="n">
-        <v>9532</v>
-      </c>
-      <c r="I17" s="6" t="n">
-        <v>9982</v>
-      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -909,29 +789,17 @@
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="B18" s="6" t="n">
-        <v>9022</v>
-      </c>
-      <c r="C18" s="6" t="n">
-        <v>12092</v>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>8272</v>
-      </c>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
       <c r="F18" s="5" t="inlineStr">
         <is>
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="G18" s="6" t="n">
-        <v>9218</v>
-      </c>
-      <c r="H18" s="6" t="n">
-        <v>9868</v>
-      </c>
-      <c r="I18" s="6" t="n">
-        <v>9878</v>
-      </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -939,29 +807,17 @@
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="B19" s="6" t="n">
-        <v>11822</v>
-      </c>
-      <c r="C19" s="6" t="n">
-        <v>11802</v>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>8872</v>
-      </c>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
       <c r="F19" s="5" t="inlineStr">
         <is>
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="G19" s="6" t="n">
-        <v>9532</v>
-      </c>
-      <c r="H19" s="6" t="n">
-        <v>10712</v>
-      </c>
-      <c r="I19" s="6" t="n">
-        <v>11088</v>
-      </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1018,29 +874,17 @@
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="B23" s="6" t="n">
-        <v>10882</v>
-      </c>
-      <c r="C23" s="6" t="n">
-        <v>10122</v>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>7422</v>
-      </c>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
       <c r="F23" s="5" t="inlineStr">
         <is>
           <t>QSRC=0</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n">
-        <v>10882</v>
-      </c>
-      <c r="H23" s="6" t="n">
-        <v>10312</v>
-      </c>
-      <c r="I23" s="6" t="n">
-        <v>8062</v>
-      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -1048,29 +892,17 @@
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="B24" s="6" t="n">
-        <v>11938</v>
-      </c>
-      <c r="C24" s="6" t="n">
-        <v>9752</v>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>5632</v>
-      </c>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
       <c r="F24" s="5" t="inlineStr">
         <is>
           <t>QSRC=1</t>
         </is>
       </c>
-      <c r="G24" s="6" t="n">
-        <v>11328</v>
-      </c>
-      <c r="H24" s="6" t="n">
-        <v>9218</v>
-      </c>
-      <c r="I24" s="6" t="n">
-        <v>5552</v>
-      </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1078,29 +910,17 @@
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n">
-        <v>10928</v>
-      </c>
-      <c r="C25" s="6" t="n">
-        <v>7902</v>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>8028</v>
-      </c>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
       <c r="F25" s="5" t="inlineStr">
         <is>
           <t>QSRC=2</t>
         </is>
       </c>
-      <c r="G25" s="6" t="n">
-        <v>9482</v>
-      </c>
-      <c r="H25" s="6" t="n">
-        <v>7628</v>
-      </c>
-      <c r="I25" s="6" t="n">
-        <v>7978</v>
-      </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -1108,29 +928,17 @@
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n">
-        <v>10178</v>
-      </c>
-      <c r="C26" s="6" t="n">
-        <v>8222</v>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>8212</v>
-      </c>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
       <c r="F26" s="5" t="inlineStr">
         <is>
           <t>QSRC=3</t>
         </is>
       </c>
-      <c r="G26" s="6" t="n">
-        <v>8318</v>
-      </c>
-      <c r="H26" s="6" t="n">
-        <v>8278</v>
-      </c>
-      <c r="I26" s="6" t="n">
-        <v>8282</v>
-      </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1138,29 +946,17 @@
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="B27" s="6" t="n">
-        <v>8258</v>
-      </c>
-      <c r="C27" s="6" t="n">
-        <v>8442</v>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>9398</v>
-      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
       <c r="F27" s="5" t="inlineStr">
         <is>
           <t>QSRC=4</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n">
-        <v>11232</v>
-      </c>
-      <c r="H27" s="6" t="n">
-        <v>8712</v>
-      </c>
-      <c r="I27" s="6" t="n">
-        <v>9178</v>
-      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -1168,29 +964,17 @@
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n">
-        <v>8648</v>
-      </c>
-      <c r="C28" s="6" t="n">
-        <v>8548</v>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>9018</v>
-      </c>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
       <c r="F28" s="5" t="inlineStr">
         <is>
           <t>QSRC=5</t>
         </is>
       </c>
-      <c r="G28" s="6" t="n">
-        <v>10338</v>
-      </c>
-      <c r="H28" s="6" t="n">
-        <v>9348</v>
-      </c>
-      <c r="I28" s="6" t="n">
-        <v>8338</v>
-      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1359,13 +1143,13 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>10238</v>
+        <v>9322</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>7568</v>
+        <v>6122</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>6148</v>
+        <v>75362</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -1373,13 +1157,13 @@
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>10238</v>
+        <v>9322</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>6102</v>
+        <v>6328</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>5118</v>
+        <v>75362</v>
       </c>
     </row>
     <row r="6">
@@ -1389,13 +1173,13 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>9088</v>
+        <v>11568</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>7358</v>
+        <v>6122</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>5342</v>
+        <v>6032</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -1403,13 +1187,13 @@
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>9872</v>
+        <v>11822</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>5752</v>
+        <v>6142</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>81248</v>
+        <v>294222</v>
       </c>
     </row>
     <row r="7">
@@ -1419,13 +1203,13 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>8858</v>
+        <v>8272</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>7732</v>
+        <v>7988</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>7682</v>
+        <v>7778</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -1433,13 +1217,13 @@
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>7698</v>
+        <v>9592</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>8018</v>
+        <v>8022</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>7782</v>
+        <v>7778</v>
       </c>
     </row>
     <row r="8">
@@ -1449,13 +1233,13 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>9092</v>
+        <v>8778</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>8062</v>
+        <v>8288</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>8038</v>
+        <v>8312</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -1463,13 +1247,13 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>8952</v>
+        <v>8802</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>8182</v>
+        <v>8342</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>8042</v>
+        <v>8218</v>
       </c>
     </row>
     <row r="9">
@@ -1479,13 +1263,13 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>8232</v>
+        <v>8772</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>8088</v>
+        <v>8328</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>8188</v>
+        <v>8342</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -1493,13 +1277,13 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>8338</v>
+        <v>8312</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>8228</v>
+        <v>8268</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>8288</v>
+        <v>8172</v>
       </c>
     </row>
     <row r="10">
@@ -1509,13 +1293,13 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>8502</v>
+        <v>10802</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>8482</v>
+        <v>8568</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>8602</v>
+        <v>8632</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -1523,13 +1307,13 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>8342</v>
+        <v>9402</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>8322</v>
+        <v>9188</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>8312</v>
+        <v>9588</v>
       </c>
     </row>
     <row r="12">
@@ -1588,13 +1372,13 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>10792</v>
+        <v>11282</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>7958</v>
+        <v>8888</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>4368</v>
+        <v>6688</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -1602,13 +1386,13 @@
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>10792</v>
+        <v>11282</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>7142</v>
+        <v>7742</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>4872</v>
+        <v>6248</v>
       </c>
     </row>
     <row r="15">
@@ -1618,13 +1402,13 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>9718</v>
+        <v>11252</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>6018</v>
+        <v>6762</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>6198</v>
+        <v>6918</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -1632,13 +1416,13 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>9652</v>
+        <v>10498</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>7212</v>
+        <v>7328</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>5952</v>
+        <v>5832</v>
       </c>
     </row>
     <row r="16">
@@ -1648,13 +1432,13 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>8448</v>
+        <v>11128</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>7728</v>
+        <v>7982</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>7662</v>
+        <v>7948</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -1662,13 +1446,13 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>9868</v>
+        <v>10328</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>7642</v>
+        <v>8172</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>7698</v>
+        <v>7858</v>
       </c>
     </row>
     <row r="17">
@@ -1678,13 +1462,13 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>8292</v>
+        <v>10922</v>
       </c>
       <c r="C17" s="6" t="n">
         <v>8332</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>8288</v>
+        <v>8202</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -1692,13 +1476,13 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>8498</v>
+        <v>8432</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>8178</v>
+        <v>8252</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>8182</v>
+        <v>8208</v>
       </c>
     </row>
     <row r="18">
@@ -1708,13 +1492,13 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>8322</v>
+        <v>9302</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>9422</v>
+        <v>8402</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>8208</v>
+        <v>10802</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -1722,13 +1506,13 @@
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>8378</v>
+        <v>9172</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>8328</v>
+        <v>8362</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>8512</v>
+        <v>8372</v>
       </c>
     </row>
     <row r="19">
@@ -1738,13 +1522,13 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>11958</v>
+        <v>9212</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>13158</v>
+        <v>8838</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>8548</v>
+        <v>9388</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -1752,13 +1536,13 @@
         </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>9132</v>
+        <v>9552</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>9368</v>
+        <v>10008</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>10038</v>
+        <v>8692</v>
       </c>
     </row>
     <row r="21">
@@ -1817,13 +1601,13 @@
         </is>
       </c>
       <c r="B23" s="6" t="n">
-        <v>11072</v>
+        <v>11082</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>10148</v>
+        <v>11432</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>8338</v>
+        <v>10522</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -1831,13 +1615,13 @@
         </is>
       </c>
       <c r="G23" s="6" t="n">
-        <v>11072</v>
+        <v>11082</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>10338</v>
+        <v>10182</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>8658</v>
+        <v>11028</v>
       </c>
     </row>
     <row r="24">
@@ -1847,13 +1631,13 @@
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>12108</v>
+        <v>12708</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>9882</v>
+        <v>11148</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>5932</v>
+        <v>6308</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1861,13 +1645,13 @@
         </is>
       </c>
       <c r="G24" s="6" t="n">
-        <v>11432</v>
+        <v>12788</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>9332</v>
+        <v>11232</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>5808</v>
+        <v>9392</v>
       </c>
     </row>
     <row r="25">
@@ -1877,13 +1661,13 @@
         </is>
       </c>
       <c r="B25" s="6" t="n">
-        <v>11018</v>
+        <v>9528</v>
       </c>
       <c r="C25" s="6" t="n">
-        <v>7912</v>
+        <v>7808</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>8108</v>
+        <v>8252</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -1891,13 +1675,13 @@
         </is>
       </c>
       <c r="G25" s="6" t="n">
-        <v>9528</v>
+        <v>10768</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>7632</v>
+        <v>8358</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>8062</v>
+        <v>8268</v>
       </c>
     </row>
     <row r="26">
@@ -1907,13 +1691,13 @@
         </is>
       </c>
       <c r="B26" s="6" t="n">
-        <v>10188</v>
+        <v>10102</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>8228</v>
+        <v>8368</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>8242</v>
+        <v>8362</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
@@ -1921,13 +1705,13 @@
         </is>
       </c>
       <c r="G26" s="6" t="n">
-        <v>8322</v>
+        <v>8862</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>8282</v>
+        <v>8962</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>8298</v>
+        <v>8358</v>
       </c>
     </row>
     <row r="27">
@@ -1937,13 +1721,13 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>8262</v>
+        <v>14382</v>
       </c>
       <c r="C27" s="6" t="n">
-        <v>8448</v>
+        <v>12868</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>9752</v>
+        <v>9058</v>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
@@ -1951,13 +1735,13 @@
         </is>
       </c>
       <c r="G27" s="6" t="n">
-        <v>11262</v>
+        <v>10642</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>8718</v>
+        <v>14552</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>9588</v>
+        <v>13978</v>
       </c>
     </row>
     <row r="28">
@@ -1967,13 +1751,13 @@
         </is>
       </c>
       <c r="B28" s="6" t="n">
-        <v>8652</v>
+        <v>10272</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>8568</v>
+        <v>10688</v>
       </c>
       <c r="D28" s="6" t="n">
-        <v>9058</v>
+        <v>14508</v>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
@@ -1981,13 +1765,13 @@
         </is>
       </c>
       <c r="G28" s="6" t="n">
-        <v>10342</v>
+        <v>10278</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>9392</v>
+        <v>9028</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>8342</v>
+        <v>15088</v>
       </c>
     </row>
   </sheetData>
@@ -2157,13 +1941,13 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>8898</v>
+        <v>8358</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>11808</v>
+        <v>11958</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>9892</v>
+        <v>9778</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
@@ -2171,13 +1955,13 @@
         </is>
       </c>
       <c r="G5" s="6" t="n">
-        <v>8898</v>
+        <v>8358</v>
       </c>
       <c r="H5" s="6" t="n">
-        <v>11552</v>
+        <v>11762</v>
       </c>
       <c r="I5" s="6" t="n">
-        <v>11102</v>
+        <v>8832</v>
       </c>
     </row>
     <row r="6">
@@ -2187,13 +1971,13 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>9618</v>
+        <v>12312</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>11818</v>
+        <v>11242</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>10438</v>
+        <v>11222</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
@@ -2201,13 +1985,13 @@
         </is>
       </c>
       <c r="G6" s="6" t="n">
-        <v>10192</v>
+        <v>11578</v>
       </c>
       <c r="H6" s="6" t="n">
-        <v>8332</v>
+        <v>10262</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>10538</v>
+        <v>11532</v>
       </c>
     </row>
     <row r="7">
@@ -2217,13 +2001,13 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>11298</v>
+        <v>11792</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>11468</v>
+        <v>13472</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>10692</v>
+        <v>11768</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
@@ -2231,13 +2015,13 @@
         </is>
       </c>
       <c r="G7" s="6" t="n">
-        <v>8318</v>
+        <v>12168</v>
       </c>
       <c r="H7" s="6" t="n">
-        <v>11972</v>
+        <v>13392</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>11212</v>
+        <v>11712</v>
       </c>
     </row>
     <row r="8">
@@ -2247,13 +2031,13 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
-        <v>11032</v>
+        <v>9838</v>
       </c>
       <c r="C8" s="6" t="n">
-        <v>8768</v>
+        <v>11822</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>9602</v>
+        <v>11688</v>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
@@ -2261,13 +2045,13 @@
         </is>
       </c>
       <c r="G8" s="6" t="n">
-        <v>11068</v>
+        <v>9978</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>10758</v>
+        <v>12558</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>10568</v>
+        <v>11052</v>
       </c>
     </row>
     <row r="9">
@@ -2277,13 +2061,13 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>9112</v>
+        <v>12178</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>8822</v>
+        <v>11078</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>10428</v>
+        <v>11632</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
@@ -2291,13 +2075,13 @@
         </is>
       </c>
       <c r="G9" s="6" t="n">
-        <v>10168</v>
+        <v>11238</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>9698</v>
+        <v>9618</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>10808</v>
+        <v>9268</v>
       </c>
     </row>
     <row r="10">
@@ -2307,13 +2091,13 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>10422</v>
+        <v>13162</v>
       </c>
       <c r="C10" s="6" t="n">
-        <v>11172</v>
+        <v>10902</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>10692</v>
+        <v>11158</v>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
@@ -2321,13 +2105,13 @@
         </is>
       </c>
       <c r="G10" s="6" t="n">
-        <v>9932</v>
+        <v>11398</v>
       </c>
       <c r="H10" s="6" t="n">
-        <v>10118</v>
+        <v>11962</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>10942</v>
+        <v>11862</v>
       </c>
     </row>
     <row r="12">
@@ -2386,13 +2170,13 @@
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>10278</v>
+        <v>10338</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>10678</v>
+        <v>11938</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>8268</v>
+        <v>10642</v>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
@@ -2400,13 +2184,13 @@
         </is>
       </c>
       <c r="G14" s="6" t="n">
-        <v>10278</v>
+        <v>10338</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>9592</v>
+        <v>10638</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>8732</v>
+        <v>10728</v>
       </c>
     </row>
     <row r="15">
@@ -2416,13 +2200,13 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>9552</v>
+        <v>12228</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>9488</v>
+        <v>12348</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>9682</v>
+        <v>12318</v>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
@@ -2430,13 +2214,13 @@
         </is>
       </c>
       <c r="G15" s="6" t="n">
-        <v>10362</v>
+        <v>10482</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>10512</v>
+        <v>12568</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>10588</v>
+        <v>8618</v>
       </c>
     </row>
     <row r="16">
@@ -2446,13 +2230,13 @@
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>9498</v>
+        <v>12228</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>9848</v>
+        <v>11342</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>9978</v>
+        <v>12292</v>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
@@ -2460,13 +2244,13 @@
         </is>
       </c>
       <c r="G16" s="6" t="n">
-        <v>11692</v>
+        <v>11698</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>10162</v>
+        <v>12758</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>10838</v>
+        <v>10612</v>
       </c>
     </row>
     <row r="17">
@@ -2476,13 +2260,13 @@
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>10242</v>
+        <v>13438</v>
       </c>
       <c r="C17" s="6" t="n">
-        <v>12678</v>
+        <v>12188</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>11742</v>
+        <v>10812</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -2490,13 +2274,13 @@
         </is>
       </c>
       <c r="G17" s="6" t="n">
-        <v>10528</v>
+        <v>11408</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>11058</v>
+        <v>11618</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>11838</v>
+        <v>12058</v>
       </c>
     </row>
     <row r="18">
@@ -2506,13 +2290,13 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>9758</v>
+        <v>10498</v>
       </c>
       <c r="C18" s="6" t="n">
-        <v>12968</v>
+        <v>10898</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>8432</v>
+        <v>12588</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
@@ -2520,13 +2304,13 @@
         </is>
       </c>
       <c r="G18" s="6" t="n">
-        <v>9968</v>
+        <v>11352</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>11102</v>
+        <v>10712</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>10752</v>
+        <v>10538</v>
       </c>
     </row>
     <row r="19">
@@ -2536,13 +2320,13 @@
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>11768</v>
+        <v>10258</v>
       </c>
       <c r="C19" s="6" t="n">
-        <v>11528</v>
+        <v>9918</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>9288</v>
+        <v>10932</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -2550,13 +2334,13 @@
         </is>
       </c>
       <c r="G19" s="6" t="n">
-        <v>9878</v>
+        <v>10572</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>11342</v>
+        <v>11098</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>11392</v>
+        <v>10348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>